<commit_message>
feat : story map
</commit_message>
<xml_diff>
--- a/docs/cadrage/equipe-02-story-map-v1.0.xlsx
+++ b/docs/cadrage/equipe-02-story-map-v1.0.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a3b0e1f223a22363/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\krimi\IPSSI_APOCAL_KIT\docs\cadrage\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{DF399E9D-FF1B-4183-8EC2-492F6C96D37D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{512D029F-2B15-493D-BF92-B176328D0871}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D2C8CD0-A030-4D17-BA54-1B11C63600F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="150">
   <si>
     <t>A</t>
   </si>
@@ -281,30 +281,17 @@
 30 s configurable)</t>
   </si>
   <si>
-    <t>US-11
-Dashboard progression par chapitre</t>
-  </si>
-  <si>
     <t>US-22
 Statistiques collectives en temps réel</t>
   </si>
   <si>
     <t>Personnalisation thème UI</t>
-  </si>
-  <si>
-    <t>US - 05
-Affiche-le score /10</t>
   </si>
   <si>
     <t>US - 06 
 Connexion
 Déconnexion
 Modifier son profil</t>
-  </si>
-  <si>
-    <t>US-12
-Export RGPD complet (JSON + CSV, Art. 
-15 / 20), lié J3-bis</t>
   </si>
   <si>
     <t>US-16
@@ -498,6 +485,49 @@
   </si>
   <si>
     <t>29/06/2026 16h50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US - 05
+Affiche-le score /10
+</t>
+  </si>
+  <si>
+    <t>US-12
+Export RGPD complet (JSON + CSV, Art. 
+15 / 20), lié J3-bis
+US-23
+Envoyer des conseils personnalisés
+aux étudiants</t>
+  </si>
+  <si>
+    <t>US-11
+Dashboard progression des étudiants
+(enseignant)
+US-22
+Consulter les scores des étudiants
+US-21
+Identifier les étudiants en difficulté</t>
+  </si>
+  <si>
+    <t>US-21</t>
+  </si>
+  <si>
+    <t>US-22</t>
+  </si>
+  <si>
+    <t>US-23</t>
+  </si>
+  <si>
+    <t>En tant qu'enseignante, je veux consulter les scores de mes étudiants afin d'identifier ceux qui ont besoin d'aide.</t>
+  </si>
+  <si>
+    <t>En tant qu'enseignante, je veux visualiser un tableau de bord de la progression de ma classe afin de suivre les performances globales.</t>
+  </si>
+  <si>
+    <t>En tant qu'enseignante, je veux envoyer des conseils de révision à mes étudiants afin de les accompagner avant les examens.</t>
+  </si>
+  <si>
+    <t>5. Consulter résultat</t>
   </si>
 </sst>
 </file>
@@ -1570,7 +1600,7 @@
         <v>13</v>
       </c>
       <c r="C9" s="22" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
     </row>
     <row r="10" spans="2:3" ht="22" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -1605,7 +1635,8 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="7" width="32" customWidth="1"/>
+    <col min="2" max="6" width="32" customWidth="1"/>
+    <col min="7" max="7" width="39.26953125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="23.5" x14ac:dyDescent="0.55000000000000004">
@@ -1673,7 +1704,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="78" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:7" ht="93.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="15" t="s">
         <v>34</v>
       </c>
@@ -1690,13 +1721,13 @@
         <v>78</v>
       </c>
       <c r="F10" s="23" t="s">
-        <v>83</v>
+        <v>140</v>
       </c>
       <c r="G10" s="23" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="139" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="16" t="s">
         <v>35</v>
       </c>
@@ -1713,10 +1744,10 @@
         <v>79</v>
       </c>
       <c r="F11" s="24" t="s">
-        <v>80</v>
+        <v>142</v>
       </c>
       <c r="G11" s="24" t="s">
-        <v>85</v>
+        <v>141</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.35">
@@ -1733,13 +1764,13 @@
         <v>77</v>
       </c>
       <c r="E12" s="25" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="F12" s="25" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="G12" s="25" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.35">
@@ -1750,19 +1781,19 @@
         <v>72</v>
       </c>
       <c r="C13" s="26" t="s">
+        <v>85</v>
+      </c>
+      <c r="D13" s="26" t="s">
+        <v>87</v>
+      </c>
+      <c r="E13" s="26" t="s">
         <v>88</v>
       </c>
-      <c r="D13" s="26" t="s">
-        <v>90</v>
-      </c>
-      <c r="E13" s="26" t="s">
-        <v>91</v>
-      </c>
       <c r="F13" s="26" t="s">
+        <v>80</v>
+      </c>
+      <c r="G13" s="26" t="s">
         <v>81</v>
-      </c>
-      <c r="G13" s="26" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.35">
@@ -1821,7 +1852,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FA14BC33-20C3-4917-AEE6-3D1546FD7916}">
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="20.453125" customWidth="1"/>
@@ -1832,24 +1863,24 @@
   <sheetData>
     <row r="1" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="39" t="s">
+        <v>109</v>
+      </c>
+      <c r="B1" s="40" t="s">
+        <v>110</v>
+      </c>
+      <c r="C1" s="40" t="s">
+        <v>111</v>
+      </c>
+      <c r="D1" s="40" t="s">
         <v>112</v>
-      </c>
-      <c r="B1" s="40" t="s">
-        <v>113</v>
-      </c>
-      <c r="C1" s="40" t="s">
-        <v>114</v>
-      </c>
-      <c r="D1" s="40" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A2" s="41" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="B2" s="42" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="C2" s="43" t="s">
         <v>39</v>
@@ -1860,10 +1891,10 @@
     </row>
     <row r="3" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A3" s="41" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="B3" s="42" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="C3" s="43" t="s">
         <v>39</v>
@@ -1874,10 +1905,10 @@
     </row>
     <row r="4" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A4" s="41" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="B4" s="42" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="C4" s="43" t="s">
         <v>39</v>
@@ -1888,10 +1919,10 @@
     </row>
     <row r="5" spans="1:4" ht="29" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A5" s="41" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="B5" s="42" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="C5" s="43" t="s">
         <v>39</v>
@@ -1902,10 +1933,10 @@
     </row>
     <row r="6" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A6" s="41" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="B6" s="42" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="C6" s="43" t="s">
         <v>39</v>
@@ -1916,10 +1947,10 @@
     </row>
     <row r="7" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A7" s="41" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="B7" s="42" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="C7" s="43" t="s">
         <v>39</v>
@@ -1930,10 +1961,10 @@
     </row>
     <row r="8" spans="1:4" ht="29" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A8" s="44" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="B8" s="45" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="C8" s="46" t="s">
         <v>41</v>
@@ -1944,10 +1975,10 @@
     </row>
     <row r="9" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A9" s="44" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="B9" s="45" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="C9" s="46" t="s">
         <v>41</v>
@@ -1958,10 +1989,10 @@
     </row>
     <row r="10" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A10" s="44" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="B10" s="45" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="C10" s="46" t="s">
         <v>41</v>
@@ -1972,10 +2003,10 @@
     </row>
     <row r="11" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A11" s="44" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="B11" s="45" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="C11" s="46" t="s">
         <v>41</v>
@@ -1986,10 +2017,10 @@
     </row>
     <row r="12" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A12" s="44" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="B12" s="45" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="C12" s="46" t="s">
         <v>41</v>
@@ -2000,127 +2031,169 @@
     </row>
     <row r="13" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A13" s="44" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="B13" s="45" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="C13" s="46" t="s">
         <v>41</v>
       </c>
       <c r="D13" s="45" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" ht="19.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A14" s="47" t="s">
-        <v>104</v>
-      </c>
-      <c r="B14" s="48" t="s">
-        <v>127</v>
-      </c>
-      <c r="C14" s="49" t="s">
-        <v>43</v>
-      </c>
-      <c r="D14" s="48" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" ht="29" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A15" s="47" t="s">
-        <v>105</v>
-      </c>
-      <c r="B15" s="48" t="s">
-        <v>128</v>
-      </c>
-      <c r="C15" s="49" t="s">
-        <v>43</v>
-      </c>
-      <c r="D15" s="48" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A16" s="47" t="s">
-        <v>106</v>
-      </c>
-      <c r="B16" s="48" t="s">
-        <v>129</v>
-      </c>
-      <c r="C16" s="49" t="s">
-        <v>43</v>
-      </c>
-      <c r="D16" s="48" t="s">
-        <v>30</v>
+        <v>123</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="25" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A14" s="44" t="s">
+        <v>143</v>
+      </c>
+      <c r="B14" s="45" t="s">
+        <v>146</v>
+      </c>
+      <c r="C14" s="46" t="s">
+        <v>41</v>
+      </c>
+      <c r="D14" s="45" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="37" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A15" s="44" t="s">
+        <v>144</v>
+      </c>
+      <c r="B15" s="45" t="s">
+        <v>147</v>
+      </c>
+      <c r="C15" s="46" t="s">
+        <v>41</v>
+      </c>
+      <c r="D15" s="45" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A16" s="44" t="s">
+        <v>145</v>
+      </c>
+      <c r="B16" s="45" t="s">
+        <v>148</v>
+      </c>
+      <c r="C16" s="46" t="s">
+        <v>41</v>
+      </c>
+      <c r="D16" s="45" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A17" s="47" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="B17" s="48" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="C17" s="49" t="s">
         <v>43</v>
       </c>
       <c r="D17" s="48" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="29" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A18" s="47" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="B18" s="48" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="C18" s="49" t="s">
         <v>43</v>
       </c>
       <c r="D18" s="48" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A19" s="47" t="s">
+        <v>103</v>
+      </c>
+      <c r="B19" s="48" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="19" spans="1:4" ht="38.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A19" s="50" t="s">
-        <v>109</v>
-      </c>
-      <c r="B19" s="51" t="s">
-        <v>132</v>
-      </c>
-      <c r="C19" s="52" t="s">
+      <c r="C19" s="49" t="s">
+        <v>43</v>
+      </c>
+      <c r="D19" s="48" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A20" s="47" t="s">
+        <v>104</v>
+      </c>
+      <c r="B20" s="48" t="s">
+        <v>127</v>
+      </c>
+      <c r="C20" s="49" t="s">
+        <v>43</v>
+      </c>
+      <c r="D20" s="48" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A21" s="47" t="s">
+        <v>105</v>
+      </c>
+      <c r="B21" s="48" t="s">
+        <v>128</v>
+      </c>
+      <c r="C21" s="49" t="s">
+        <v>43</v>
+      </c>
+      <c r="D21" s="48" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" ht="38.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A22" s="50" t="s">
+        <v>106</v>
+      </c>
+      <c r="B22" s="51" t="s">
+        <v>129</v>
+      </c>
+      <c r="C22" s="52" t="s">
         <v>45</v>
       </c>
-      <c r="D19" s="51" t="s">
+      <c r="D22" s="51" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="20" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A20" s="50" t="s">
-        <v>110</v>
-      </c>
-      <c r="B20" s="51" t="s">
-        <v>133</v>
-      </c>
-      <c r="C20" s="52" t="s">
+    <row r="23" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A23" s="50" t="s">
+        <v>107</v>
+      </c>
+      <c r="B23" s="51" t="s">
+        <v>130</v>
+      </c>
+      <c r="C23" s="52" t="s">
         <v>45</v>
       </c>
-      <c r="D20" s="51" t="s">
+      <c r="D23" s="51" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="21" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A21" s="50" t="s">
-        <v>111</v>
-      </c>
-      <c r="B21" s="51" t="s">
-        <v>134</v>
-      </c>
-      <c r="C21" s="52" t="s">
+    <row r="24" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A24" s="50" t="s">
+        <v>108</v>
+      </c>
+      <c r="B24" s="51" t="s">
+        <v>131</v>
+      </c>
+      <c r="C24" s="52" t="s">
         <v>45</v>
       </c>
-      <c r="D21" s="51" t="s">
+      <c r="D24" s="51" t="s">
         <v>31</v>
       </c>
     </row>
@@ -2168,10 +2241,10 @@
         <v>54</v>
       </c>
       <c r="C6" s="53" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="D6" s="56" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="44" customHeight="1" x14ac:dyDescent="0.35">
@@ -2179,10 +2252,10 @@
         <v>55</v>
       </c>
       <c r="C7" s="53" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="D7" s="56" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.35">
@@ -2190,7 +2263,7 @@
         <v>56</v>
       </c>
       <c r="C8" s="53" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="D8" s="56"/>
     </row>
@@ -2199,7 +2272,7 @@
         <v>57</v>
       </c>
       <c r="C9" s="53" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="D9" s="56"/>
     </row>
@@ -2208,7 +2281,7 @@
         <v>58</v>
       </c>
       <c r="C10" s="53" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="D10" s="56"/>
     </row>
@@ -2217,7 +2290,7 @@
         <v>59</v>
       </c>
       <c r="C11" s="53" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="D11" s="56"/>
     </row>
@@ -2226,10 +2299,10 @@
         <v>60</v>
       </c>
       <c r="C12" s="53" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="D12" s="54" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.35">
@@ -2237,7 +2310,7 @@
         <v>61</v>
       </c>
       <c r="C13" s="53" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="D13" s="56"/>
     </row>
@@ -2246,10 +2319,10 @@
         <v>62</v>
       </c>
       <c r="C14" s="53" t="s">
+        <v>134</v>
+      </c>
+      <c r="D14" s="56" t="s">
         <v>137</v>
-      </c>
-      <c r="D14" s="56" t="s">
-        <v>140</v>
       </c>
     </row>
   </sheetData>

</xml_diff>